<commit_message>
le simulateur Excel ne fusionne plus de cellule seule sur le tableau de bord, ce qui faisait planter Numbers à l'ouverture
</commit_message>
<xml_diff>
--- a/docs/tarification/simulateur-tarification.xlsx
+++ b/docs/tarification/simulateur-tarification.xlsx
@@ -1830,29 +1830,24 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="23">
+  <mergeCells count="18">
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F23:H23"/>
     <mergeCell ref="G12:H12"/>
+    <mergeCell ref="F19:H19"/>
     <mergeCell ref="F21:H21"/>
+    <mergeCell ref="B17:C18"/>
+    <mergeCell ref="E10:F10"/>
     <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="B68:H68"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="E16"/>
     <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="E18"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="E17"/>
-    <mergeCell ref="E20"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E19"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="B17:C18"/>
     <mergeCell ref="F15:H15"/>
   </mergeCells>
   <conditionalFormatting sqref="C16">

</xml_diff>